<commit_message>
fix tecnologia terceiro eth
</commit_message>
<xml_diff>
--- a/arquivos/facilidades_tecnologia_prioridade.xlsx
+++ b/arquivos/facilidades_tecnologia_prioridade.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\F257064\Documents\Codes\atualizacao automacao lote\AUTMACAO_LOTE\arquivos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD1425E2-A492-495C-ABE5-F6B11C30A6B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1ADF764-C8F8-4021-BA83-5A879A5032D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -179,7 +179,7 @@
     <t>XGSPON RES MOVEL</t>
   </si>
   <si>
-    <t>TERCEIROS ETH</t>
+    <t>TERCEIRO ETH</t>
   </si>
 </sst>
 </file>

</xml_diff>